<commit_message>
changed time to 24hr format
</commit_message>
<xml_diff>
--- a/OpenVPM/src/test/resources/testData.xlsx
+++ b/OpenVPM/src/test/resources/testData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\git\repositoryOpenVpm\OpenVPM\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{211F66F4-3B1B-4A6E-87B3-EB40F34BFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCF29B46-71EC-4FFA-9E03-4F4964EC5AD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Clients" sheetId="1" r:id="rId1"/>
@@ -489,18 +489,6 @@
     <t>Gregory</t>
   </si>
   <si>
-    <t>01:00</t>
-  </si>
-  <si>
-    <t>01:30</t>
-  </si>
-  <si>
-    <t>02:00</t>
-  </si>
-  <si>
-    <t>02:30</t>
-  </si>
-  <si>
     <t>Exam Room 3</t>
   </si>
   <si>
@@ -528,24 +516,6 @@
     <t>VacciBordetella</t>
   </si>
   <si>
-    <t>03:30</t>
-  </si>
-  <si>
-    <t>03:00</t>
-  </si>
-  <si>
-    <t>04:00</t>
-  </si>
-  <si>
-    <t>04:30</t>
-  </si>
-  <si>
-    <t>05:00</t>
-  </si>
-  <si>
-    <t>05:30</t>
-  </si>
-  <si>
     <t>Exam Room 4</t>
   </si>
   <si>
@@ -556,6 +526,36 @@
   </si>
   <si>
     <t>Exam Room 7</t>
+  </si>
+  <si>
+    <t>13:00</t>
+  </si>
+  <si>
+    <t>13:30</t>
+  </si>
+  <si>
+    <t>14:00</t>
+  </si>
+  <si>
+    <t>14:30</t>
+  </si>
+  <si>
+    <t>15:00</t>
+  </si>
+  <si>
+    <t>15:30</t>
+  </si>
+  <si>
+    <t>16:00</t>
+  </si>
+  <si>
+    <t>16:30</t>
+  </si>
+  <si>
+    <t>17:00</t>
+  </si>
+  <si>
+    <t>17:30</t>
   </si>
 </sst>
 </file>
@@ -611,13 +611,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1099,10 +1098,10 @@
         <v>92</v>
       </c>
       <c r="G1" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>158</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
@@ -1125,10 +1124,10 @@
         <v>116</v>
       </c>
       <c r="G2" t="s">
+        <v>155</v>
+      </c>
+      <c r="H2" t="s">
         <v>159</v>
-      </c>
-      <c r="H2" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1151,10 +1150,10 @@
         <v>117</v>
       </c>
       <c r="G3" t="s">
+        <v>156</v>
+      </c>
+      <c r="H3" t="s">
         <v>160</v>
-      </c>
-      <c r="H3" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
@@ -1177,10 +1176,10 @@
         <v>118</v>
       </c>
       <c r="G4" t="s">
+        <v>157</v>
+      </c>
+      <c r="H4" t="s">
         <v>161</v>
-      </c>
-      <c r="H4" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
@@ -1481,7 +1480,7 @@
         <v>13</v>
       </c>
       <c r="D6" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>26</v>
@@ -1492,7 +1491,7 @@
         <v>14</v>
       </c>
       <c r="D7" t="s">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>27</v>
@@ -1500,7 +1499,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="D8" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>28</v>
@@ -1508,7 +1507,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="D9" t="s">
-        <v>174</v>
+        <v>164</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>149</v>
@@ -1516,7 +1515,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="D10" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>150</v>
@@ -1529,52 +1528,52 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="E12" s="2" t="s">
-        <v>153</v>
+        <v>166</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="E13" s="2" t="s">
-        <v>154</v>
+        <v>167</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="E14" s="2" t="s">
-        <v>155</v>
+        <v>168</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="E15" s="5" t="s">
-        <v>156</v>
+      <c r="E15" s="2" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="E16" s="5" t="s">
-        <v>167</v>
+      <c r="E16" s="2" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="17" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E17" s="5" t="s">
-        <v>166</v>
+      <c r="E17" s="2" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="18" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E18" s="5" t="s">
-        <v>168</v>
+      <c r="E18" s="2" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="19" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E19" s="5" t="s">
-        <v>169</v>
+      <c r="E19" s="2" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="20" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E20" s="5" t="s">
-        <v>170</v>
+      <c r="E20" s="2" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="21" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E21" s="5" t="s">
-        <v>171</v>
+      <c r="E21" s="2" t="s">
+        <v>175</v>
       </c>
     </row>
   </sheetData>

</xml_diff>